<commit_message>
absence counting, teachers payments and forfeiture absence logic update
</commit_message>
<xml_diff>
--- a/data/attendance/ECOLE/ECOLE_فردي_تسيير_واقتصاد.xlsx
+++ b/data/attendance/ECOLE/ECOLE_فردي_تسيير_واقتصاد.xlsx
@@ -1,40 +1,121 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448B48F8-8B81-450B-93F9-1E2170FD7E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Présences" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="📖 Instructions" state="visible" r:id="rId5"/>
+    <sheet name="Présences" sheetId="1" r:id="rId1"/>
+    <sheet name="📖 Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="B5" authorId="0">
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>student_id:06d53874-9e78-4fb3-adf1-34203efd9b8c</t>
         </r>
       </text>
     </comment>
-    <comment ref="B6" authorId="0">
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>student_id:03e40222-f46d-4d70-8d16-0ab2aa5b7374</t>
         </r>
       </text>
     </comment>
-    <comment ref="B7" authorId="0">
+    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>student_id:5c8def97-b770-40ae-a2cf-7326e91ee041</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>student_id:1b3e7477-f256-4828-a3c2-495b20b37728</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>student_id:893553bd-124b-41ba-8fb7-2b0511a36128</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>student_id:602a1af7-c713-4a3e-844c-a706e64d7aad</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>student_id:3de4a94a-ad43-475f-99db-79f836b5d373</t>
         </r>
       </text>
     </comment>
@@ -43,7 +124,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
   <si>
     <t>فردي تسيير واقتصاد  |  ECOLE  |  BAC  |  خلود فردي</t>
   </si>
@@ -66,9 +147,6 @@
     <t>الاسم واللقب</t>
   </si>
   <si>
-    <t>05/09/2026</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -79,6 +157,18 @@
   </si>
   <si>
     <t>دزيري يحي</t>
+  </si>
+  <si>
+    <t>كشتولي محمد أرسلان</t>
+  </si>
+  <si>
+    <t>بهاز كوثر</t>
+  </si>
+  <si>
+    <t>بليلي ميار</t>
+  </si>
+  <si>
+    <t>بوعروج لؤي+محمد</t>
   </si>
   <si>
     <t>تعليمات ملء الحضور والكتب / Instructions</t>
@@ -117,46 +207,53 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="9"/>
       <color rgb="FFC00000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFC00000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="666666"/>
-      <sz val="9"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="9">
@@ -229,14 +326,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -259,6 +350,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,34 +697,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="14" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" hidden="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+    </row>
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -635,221 +735,397 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0</v>
-      </c>
-      <c r="K3" s="3">
-        <v>0</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3">
-        <v>0</v>
-      </c>
-      <c r="N3" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="1">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="C4" s="11">
+        <v>46284</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>63</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
-        <v>63</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0</v>
+      </c>
+      <c r="M5" s="6">
+        <v>0</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>203</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="8">
-        <v>0</v>
-      </c>
-      <c r="D5" s="8">
-        <v>0</v>
-      </c>
-      <c r="E5" s="8">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8">
-        <v>0</v>
-      </c>
-      <c r="G5" s="8">
-        <v>0</v>
-      </c>
-      <c r="H5" s="8">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8">
-        <v>0</v>
-      </c>
-      <c r="K5" s="8">
-        <v>0</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0</v>
-      </c>
-      <c r="M5" s="8">
-        <v>0</v>
-      </c>
-      <c r="N5" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <v>203</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7">
+        <v>0</v>
+      </c>
+      <c r="M6" s="7">
+        <v>0</v>
+      </c>
+      <c r="N6" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>204</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9">
-        <v>0</v>
-      </c>
-      <c r="D6" s="9">
-        <v>0</v>
-      </c>
-      <c r="E6" s="9">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9">
-        <v>0</v>
-      </c>
-      <c r="G6" s="9">
-        <v>0</v>
-      </c>
-      <c r="H6" s="9">
-        <v>0</v>
-      </c>
-      <c r="I6" s="9">
-        <v>0</v>
-      </c>
-      <c r="J6" s="9">
-        <v>0</v>
-      </c>
-      <c r="K6" s="9">
-        <v>0</v>
-      </c>
-      <c r="L6" s="9">
-        <v>0</v>
-      </c>
-      <c r="M6" s="9">
-        <v>0</v>
-      </c>
-      <c r="N6" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
-        <v>204</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
+        <v>0</v>
+      </c>
+      <c r="M7" s="6">
+        <v>0</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>286</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8">
-        <v>0</v>
-      </c>
-      <c r="J7" s="8">
-        <v>0</v>
-      </c>
-      <c r="K7" s="8">
-        <v>0</v>
-      </c>
-      <c r="L7" s="8">
-        <v>0</v>
-      </c>
-      <c r="M7" s="8">
-        <v>0</v>
-      </c>
-      <c r="N7" s="8">
+      <c r="C8" s="7">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>335</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="6">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6">
+        <v>0</v>
+      </c>
+      <c r="N9" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>336</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7">
+        <v>0</v>
+      </c>
+      <c r="F10" s="7">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7">
+        <v>0</v>
+      </c>
+      <c r="H10" s="7">
+        <v>0</v>
+      </c>
+      <c r="I10" s="7">
+        <v>0</v>
+      </c>
+      <c r="J10" s="7">
+        <v>0</v>
+      </c>
+      <c r="K10" s="7">
+        <v>0</v>
+      </c>
+      <c r="L10" s="7">
+        <v>0</v>
+      </c>
+      <c r="M10" s="7">
+        <v>0</v>
+      </c>
+      <c r="N10" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>337</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="6">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
+        <v>0</v>
+      </c>
+      <c r="M11" s="6">
+        <v>0</v>
+      </c>
+      <c r="N11" s="6">
         <v>0</v>
       </c>
     </row>
@@ -859,99 +1135,99 @@
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
-        <v>12</v>
+    <row r="1" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>